<commit_message>
add user active status
</commit_message>
<xml_diff>
--- a/data/ADS_data.xlsx
+++ b/data/ADS_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\devwork\0_ZYU_assessment_tool\ADS4\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8EC1C98-B777-4CC5-855D-19E1EB20B314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABFCF0D-9C01-4A57-9753-FDA53F412392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29660" windowHeight="18620" activeTab="3" xr2:uid="{B02D34BA-A3EF-46EF-AC77-45ABA8DC269E}"/>
+    <workbookView xWindow="4200" yWindow="1400" windowWidth="22080" windowHeight="13510" activeTab="3" xr2:uid="{B02D34BA-A3EF-46EF-AC77-45ABA8DC269E}"/>
   </bookViews>
   <sheets>
     <sheet name="Courses" sheetId="2" r:id="rId1"/>
@@ -1145,6 +1145,7 @@
   <dimension ref="A1:F53"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.90625" bestFit="1" customWidth="1"/>

</xml_diff>